<commit_message>
fix(workpaper-sync): 第二批权威模板 43 格公式错误修正，前端按模板对齐 D1-7 / 变动率 / 坏账减值明细 / F3-1 G3-1 G10-1（oo-writeback-template-parity-closure 第二批）
模板（scripts/fix/fix_template_formula_defects.py #20~#28，6 本 43 格）：
- D1-1 银行承兑汇票期初取了 D1-2 合计行；D1-15 ④ 改回录入格（原为 ①−③ 致 ⑤ 恒为 2×③−①）
- D2-9 单项区差异 B−E → D−E、小计行两格互换；D2-3 组合区小计漏 R21、期末审定漏重分类；D2-10 C90 取到表外
- D7-6 合同负债期末改贷方方向；D7-1 小计区间多含表头行；G10-1 / G13-1 引错行
- 契约 6 份、模板快照、预填定位表、D / G slice、golden、变异锚点随之重算；D1-4 G/J 两列映射改按加减方向

前端按修正后模板对齐：
- D1-7 备查簿 Q~W 由模板公式派生只读、状态取值按模板、核对表与未到期汇总按模板重做
- 变动率期初为 0 统一按模板（templateChangeRate.ts），D1~D7 / F1 / F4 审定表
- D1-4 / D2-3 / D6-3 坏账减值明细与 F3-1 / G3-1 / G10-1 期末未审从期初未审起算；D2-3 两列原绑不存在的字段（录入恒丢）
- D1-15 / D2-9 差异改为 应计提 − 账面；F4-6 期末按模板、核对来源取 F4-2 期末余额
- 顺带修 F3 信用证类别崩溃（f2d7334ac 引入）

回归：后端全量对第一批基线由过转红 0；前端全量对 13120d6d6 由过转红 1（a173 随机用例，单跑通过）。
真实项目未重发布（和平 2024 / 2025、重药安徽 2025，见 design §2）。
</commit_message>
<xml_diff>
--- a/backend/wp_templates/D/D1 应收票据.xlsx
+++ b/backend/wp_templates/D/D1 应收票据.xlsx
@@ -16071,8 +16071,10 @@
       <c r="D13" s="18" t="s">
         <v>548</v>
       </c>
-      <c r="E13" s="18" t="s">
-        <v>549</v>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
       </c>
       <c r="F13" s="18" t="s">
         <v>550</v>
@@ -16088,10 +16090,7 @@
         <f>B14*C14</f>
         <v>0</v>
       </c>
-      <c r="E14" s="23">
-        <f>B14-D14</f>
-        <v>0</v>
-      </c>
+      <c r="E14" s="23"/>
       <c r="F14" s="23">
         <f>D14-E14</f>
         <v>0</v>
@@ -16107,10 +16106,7 @@
         <f>B15*C15</f>
         <v>0</v>
       </c>
-      <c r="E15" s="23">
-        <f t="shared" ref="E15:E17" si="0">B15-D15</f>
-        <v>0</v>
-      </c>
+      <c r="E15" s="23"/>
       <c r="F15" s="23">
         <f t="shared" ref="F15:F17" si="1">D15-E15</f>
         <v>0</v>
@@ -16126,10 +16122,7 @@
         <f t="shared" ref="D16:D17" si="2">B16*C16</f>
         <v>0</v>
       </c>
-      <c r="E16" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="E16" s="23"/>
       <c r="F16" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -16145,10 +16138,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E17" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="E17" s="23"/>
       <c r="F17" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -16229,8 +16219,10 @@
       <c r="D21" s="18" t="s">
         <v>548</v>
       </c>
-      <c r="E21" s="18" t="s">
-        <v>549</v>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
       </c>
       <c r="F21" s="18" t="s">
         <v>550</v>
@@ -16248,10 +16240,7 @@
         <f>B22*C22</f>
         <v>0</v>
       </c>
-      <c r="E22" s="37">
-        <f>B22-D22</f>
-        <v>0</v>
-      </c>
+      <c r="E22" s="37"/>
       <c r="F22" s="37">
         <f>D22-E22</f>
         <v>0</v>
@@ -16269,10 +16258,7 @@
         <f>B23*C23</f>
         <v>0</v>
       </c>
-      <c r="E23" s="37">
-        <f>B23-D23</f>
-        <v>0</v>
-      </c>
+      <c r="E23" s="37"/>
       <c r="F23" s="37">
         <f t="shared" ref="F23:F24" si="3">D23-E23</f>
         <v>0</v>
@@ -16290,10 +16276,7 @@
         <f>B24*C24</f>
         <v>0</v>
       </c>
-      <c r="E24" s="37">
-        <f>B24-D24</f>
-        <v>0</v>
-      </c>
+      <c r="E24" s="37"/>
       <c r="F24" s="37">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -17897,15 +17880,15 @@
         <v>126</v>
       </c>
       <c r="B8" s="543">
-        <f>'原值明细表（按类别）D1-2'!B14</f>
+        <f>'原值明细表（按类别）D1-2'!B11</f>
         <v>0</v>
       </c>
       <c r="C8" s="543">
-        <f>'原值明细表（按类别）D1-2'!C14</f>
+        <f>'原值明细表（按类别）D1-2'!C11</f>
         <v>0</v>
       </c>
       <c r="D8" s="543">
-        <f>'原值明细表（按类别）D1-2'!D14</f>
+        <f>'原值明细表（按类别）D1-2'!D11</f>
         <v>0</v>
       </c>
       <c r="E8" s="544">

</xml_diff>